<commit_message>
fix: apply Monday Day = 0 and standard factory norms to Excel plan and DB
</commit_message>
<xml_diff>
--- a/monthly_plan_board_v2.xlsx
+++ b/monthly_plan_board_v2.xlsx
@@ -468,7 +468,7 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>1271</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr"/>
     </row>
@@ -492,7 +492,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F3" t="inlineStr"/>
     </row>
@@ -516,7 +516,7 @@
         <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F4" t="inlineStr"/>
     </row>
@@ -540,7 +540,7 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F5" t="inlineStr"/>
     </row>
@@ -564,7 +564,7 @@
         <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F6" t="inlineStr"/>
     </row>
@@ -588,7 +588,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F7" t="inlineStr"/>
     </row>
@@ -612,7 +612,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F8" t="inlineStr"/>
     </row>
@@ -636,7 +636,7 @@
         <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
@@ -660,7 +660,7 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F10" t="inlineStr"/>
     </row>
@@ -684,7 +684,7 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F11" t="inlineStr"/>
     </row>
@@ -708,7 +708,7 @@
         <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F12" t="inlineStr"/>
     </row>
@@ -732,7 +732,7 @@
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F13" t="inlineStr"/>
     </row>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F14" t="inlineStr"/>
     </row>
@@ -780,7 +780,7 @@
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F15" t="inlineStr"/>
     </row>
@@ -804,7 +804,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>1271</v>
+        <v>0</v>
       </c>
       <c r="F16" t="inlineStr"/>
     </row>
@@ -828,7 +828,7 @@
         <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F17" t="inlineStr"/>
     </row>
@@ -852,7 +852,7 @@
         <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F18" t="inlineStr"/>
     </row>
@@ -876,7 +876,7 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F19" t="inlineStr"/>
     </row>
@@ -900,7 +900,7 @@
         <v>4</v>
       </c>
       <c r="E20" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F20" t="inlineStr"/>
     </row>
@@ -924,7 +924,7 @@
         <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F21" t="inlineStr"/>
     </row>
@@ -948,7 +948,7 @@
         <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F22" t="inlineStr"/>
     </row>
@@ -972,7 +972,7 @@
         <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F23" t="inlineStr"/>
     </row>
@@ -996,7 +996,7 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F24" t="inlineStr"/>
     </row>
@@ -1020,7 +1020,7 @@
         <v>2</v>
       </c>
       <c r="E25" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F25" t="inlineStr"/>
     </row>
@@ -1044,7 +1044,7 @@
         <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F26" t="inlineStr"/>
     </row>
@@ -1068,7 +1068,7 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F27" t="inlineStr"/>
     </row>
@@ -1092,7 +1092,7 @@
         <v>4</v>
       </c>
       <c r="E28" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F28" t="inlineStr"/>
     </row>
@@ -1116,7 +1116,7 @@
         <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F29" t="inlineStr"/>
     </row>
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>1271</v>
+        <v>0</v>
       </c>
       <c r="F30" t="inlineStr"/>
     </row>
@@ -1164,7 +1164,7 @@
         <v>4</v>
       </c>
       <c r="E31" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F31" t="inlineStr"/>
     </row>
@@ -1188,7 +1188,7 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F32" t="inlineStr"/>
     </row>
@@ -1212,7 +1212,7 @@
         <v>2</v>
       </c>
       <c r="E33" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F33" t="inlineStr"/>
     </row>
@@ -1236,7 +1236,7 @@
         <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F34" t="inlineStr"/>
     </row>
@@ -1260,7 +1260,7 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F35" t="inlineStr"/>
     </row>
@@ -1284,7 +1284,7 @@
         <v>4</v>
       </c>
       <c r="E36" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F36" t="inlineStr"/>
     </row>
@@ -1308,7 +1308,7 @@
         <v>3</v>
       </c>
       <c r="E37" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F37" t="inlineStr"/>
     </row>
@@ -1332,7 +1332,7 @@
         <v>2</v>
       </c>
       <c r="E38" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F38" t="inlineStr"/>
     </row>
@@ -1356,7 +1356,7 @@
         <v>4</v>
       </c>
       <c r="E39" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>
@@ -1380,7 +1380,7 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F40" t="inlineStr"/>
     </row>
@@ -1404,7 +1404,7 @@
         <v>2</v>
       </c>
       <c r="E41" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F41" t="inlineStr"/>
     </row>
@@ -1428,7 +1428,7 @@
         <v>3</v>
       </c>
       <c r="E42" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F42" t="inlineStr"/>
     </row>
@@ -1452,7 +1452,7 @@
         <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>
@@ -1476,7 +1476,7 @@
         <v>4</v>
       </c>
       <c r="E44" t="n">
-        <v>1271</v>
+        <v>0</v>
       </c>
       <c r="F44" t="inlineStr"/>
     </row>
@@ -1500,7 +1500,7 @@
         <v>3</v>
       </c>
       <c r="E45" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F45" t="inlineStr"/>
     </row>
@@ -1524,7 +1524,7 @@
         <v>2</v>
       </c>
       <c r="E46" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F46" t="inlineStr"/>
     </row>
@@ -1548,7 +1548,7 @@
         <v>4</v>
       </c>
       <c r="E47" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F47" t="inlineStr"/>
     </row>
@@ -1572,7 +1572,7 @@
         <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F48" t="inlineStr"/>
     </row>
@@ -1596,7 +1596,7 @@
         <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F49" t="inlineStr"/>
     </row>
@@ -1620,7 +1620,7 @@
         <v>3</v>
       </c>
       <c r="E50" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F50" t="inlineStr"/>
     </row>
@@ -1644,7 +1644,7 @@
         <v>1</v>
       </c>
       <c r="E51" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F51" t="inlineStr"/>
     </row>
@@ -1668,7 +1668,7 @@
         <v>4</v>
       </c>
       <c r="E52" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F52" t="inlineStr"/>
     </row>
@@ -1692,7 +1692,7 @@
         <v>3</v>
       </c>
       <c r="E53" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F53" t="inlineStr"/>
     </row>
@@ -1716,7 +1716,7 @@
         <v>2</v>
       </c>
       <c r="E54" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F54" t="inlineStr"/>
     </row>
@@ -1740,7 +1740,7 @@
         <v>4</v>
       </c>
       <c r="E55" t="n">
-        <v>3003</v>
+        <v>3300</v>
       </c>
       <c r="F55" t="inlineStr"/>
     </row>
@@ -1764,7 +1764,7 @@
         <v>1</v>
       </c>
       <c r="E56" t="n">
-        <v>2542</v>
+        <v>2700</v>
       </c>
       <c r="F56" t="inlineStr"/>
     </row>
@@ -1788,7 +1788,7 @@
         <v>2</v>
       </c>
       <c r="E57" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F57" t="inlineStr"/>
     </row>
@@ -1812,7 +1812,7 @@
         <v>3</v>
       </c>
       <c r="E58" t="n">
-        <v>1270</v>
+        <v>0</v>
       </c>
       <c r="F58" t="inlineStr"/>
     </row>
@@ -1836,7 +1836,7 @@
         <v>1</v>
       </c>
       <c r="E59" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F59" t="inlineStr"/>
     </row>
@@ -1860,7 +1860,7 @@
         <v>4</v>
       </c>
       <c r="E60" t="n">
-        <v>2541</v>
+        <v>2700</v>
       </c>
       <c r="F60" t="inlineStr"/>
     </row>
@@ -1884,7 +1884,7 @@
         <v>3</v>
       </c>
       <c r="E61" t="n">
-        <v>3004</v>
+        <v>3300</v>
       </c>
       <c r="F61" t="inlineStr"/>
     </row>

</xml_diff>